<commit_message>
chore: regenerate the department example workbook
</commit_message>
<xml_diff>
--- a/ejemplos-generados/gestion-departamento.xlsx
+++ b/ejemplos-generados/gestion-departamento.xlsx
@@ -717,7 +717,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>07/09/2026 16:52</t>
+          <t>07/09/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
   <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="29" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>

</xml_diff>